<commit_message>
Re-run DIS AAPL JNJ NVDA ADBE WMT with latest engine
Key changes picked up:
- Rule 21 historical EV/EBITDA anchoring (EM multiples corrected):
  DIS 10x->16.1x, AAPL 10x->18.4x, JNJ 10x->20x, NVDA capped 28x,
  ADBE 15x->23.3x, WMT 10x->15x
- WACC floor 8.5%: JNJ (raw 7.0%->floored), WMT (raw 8.0%->floored)
- Forward P/E now used for scoring (analyst consensus)
- Credit ratings auto-feed (WACC cost-of-debt from agency ratings)
- Score changes: DIS +1.3, NVDA +0.3, ADBE +0.1, WMT +0.2, AAPL -0.1, JNJ -0.1

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/AAPL_model.xlsx
+++ b/static/excel/AAPL_model.xlsx
@@ -7344,11 +7344,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>4535749.27992</v>
+        <v>4557486.387511</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $308.82</t>
+          <t>FMP marketCap  |  price $310.29999</t>
         </is>
       </c>
     </row>
@@ -7659,25 +7659,27 @@
       </c>
       <c r="B32" s="53" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>AA+</t>
         </is>
       </c>
       <c r="C32" s="44" t="inlineStr">
         <is>
-          <t>FMP /ratings endpoint</t>
+          <t>User input</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>FRED matched yield</t>
-        </is>
-      </c>
-      <c r="B33" s="53" t="n"/>
+          <t>FRED matched yield  (rating-tier index)</t>
+        </is>
+      </c>
+      <c r="B33" s="46" t="n">
+        <v>0.04969999999999999</v>
+      </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>No rating returned — FRED method not applicable</t>
+          <t>FRED BAMLC0A2CAAEY — AA</t>
         </is>
       </c>
     </row>
@@ -7748,11 +7750,11 @@
         </is>
       </c>
       <c r="B38" s="48" t="n">
-        <v>0.0256</v>
+        <v>0.0336</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
-          <t>Default = average of 2 source(s) above — override freely</t>
+          <t>Default = average of 3 source(s) above — override freely</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8586,7 @@
       </c>
       <c r="J16" s="82" t="inlineStr">
         <is>
-          <t>574,307 — 633,968</t>
+          <t>466,391 — 514,842</t>
         </is>
       </c>
       <c r="K16" s="82" t="inlineStr">
@@ -8782,7 +8784,7 @@
       </c>
       <c r="J21" s="82" t="inlineStr">
         <is>
-          <t>207,288 — 228,821</t>
+          <t>168,337 — 185,824</t>
         </is>
       </c>
       <c r="K21" s="82" t="inlineStr">
@@ -9451,7 +9453,7 @@
         </is>
       </c>
       <c r="B38" s="100" t="n">
-        <v>10</v>
+        <v>18.4</v>
       </c>
       <c r="C38" s="98" t="n"/>
       <c r="D38" s="98" t="n"/>
@@ -9465,7 +9467,7 @@
       <c r="L38" s="98" t="n"/>
       <c r="M38" s="74" t="inlineStr">
         <is>
-          <t>Growth tier: LOW (1.9% 3yr avg rev growth).  Bear 8x / Base 10x / Bull 12x.  Override manually if needed.</t>
+          <t>Growth tier: LOW (1.9% 3yr avg rev growth).  Bear 15x / Base 18x / Bull 22x.  Override manually if needed.</t>
         </is>
       </c>
     </row>
@@ -9967,7 +9969,7 @@
         </is>
       </c>
       <c r="B61" s="111" t="n">
-        <v>308.82</v>
+        <v>310.3</v>
       </c>
       <c r="C61" s="103" t="n"/>
       <c r="D61" s="103" t="n"/>
@@ -10067,7 +10069,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="113" t="inlineStr">
         <is>
-          <t>JS SCORECARD — AAPL  |  Master Prompt v2  |  24 May 2026  |  Sector bucket: Tech Growth</t>
+          <t>JS SCORECARD — AAPL  |  Master Prompt v2  |  26 May 2026  |  Sector bucket: Tech Growth</t>
         </is>
       </c>
     </row>
@@ -10584,7 +10586,7 @@
       </c>
       <c r="D22" s="129" t="inlineStr">
         <is>
-          <t>Current 34.1x  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.1x [ref only — not used as benchmark]  [+14% vs benchmark]  [trail=4.75 | fwd_pe=35.3x→4.11 | abs=4.0 → blended 40/40/20=4.35]  PEG=210.90 (fwd_pe=35.3x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
+          <t>Fwd P/E 35.5x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.0x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=4.00 | fwd_pe=35.5x→4.00 | abs=1.5 → blended 40/40/20=3.50]  PEG=212.09 (fwd_pe=35.5x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
         </is>
       </c>
       <c r="E22" s="136" t="inlineStr">
@@ -10593,7 +10595,7 @@
         </is>
       </c>
       <c r="F22" s="131" t="n">
-        <v>4.6</v>
+        <v>3.75</v>
       </c>
       <c r="G22" s="132">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10601,7 +10603,7 @@
       </c>
       <c r="H22" s="133" t="inlineStr">
         <is>
-          <t>Current 34.1x  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.1x [ref only — not used as benchmark]  [+14% vs benchmark]  [trail=4.75 | fwd_pe=35.3x→4.11 | abs=4.0 → blended 40/40/20=4.35]  PEG=210.90 (fwd_pe=35.3x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
+          <t>Fwd P/E 35.5x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.0x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=4.00 | fwd_pe=35.5x→4.00 | abs=1.5 → blended 40/40/20=3.50]  PEG=212.09 (fwd_pe=35.5x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10623,7 @@
       </c>
       <c r="D23" s="129" t="inlineStr">
         <is>
-          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.8x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=40.8x→0.20 | abs=4.0 → blended 40/40/20=1.32]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
+          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.7x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=41.0x→0.11 | abs=4.0 → blended 40/40/20=1.29]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
         </is>
       </c>
       <c r="E23" s="134" t="inlineStr">
@@ -10630,7 +10632,7 @@
         </is>
       </c>
       <c r="F23" s="131" t="n">
-        <v>1.07</v>
+        <v>1.04</v>
       </c>
       <c r="G23" s="132">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10638,7 +10640,7 @@
       </c>
       <c r="H23" s="133" t="inlineStr">
         <is>
-          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.8x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=40.8x→0.20 | abs=4.0 → blended 40/40/20=1.32]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
+          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.7x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=41.0x→0.11 | abs=4.0 → blended 40/40/20=1.29]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-run DIS AAPL JNJ NVDA ADBE WMT COST NKE with latest engine
Refreshes the 8 oldest dashboard tickers (prev run 2026-05-26) on live prices.
Scores stable: AAPL +0.1, NKE -0.1, others flat.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/AAPL_model.xlsx
+++ b/static/excel/AAPL_model.xlsx
@@ -7344,11 +7344,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>4557486.387511</v>
+        <v>4589945.62356</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $310.29999</t>
+          <t>FMP marketCap  |  price $312.51</t>
         </is>
       </c>
     </row>
@@ -7430,11 +7430,11 @@
         </is>
       </c>
       <c r="B12" s="46" t="n">
-        <v>0.0457</v>
+        <v>0.043</v>
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-21</t>
+          <t>FRED series DGS10  |  latest: None</t>
         </is>
       </c>
     </row>
@@ -7445,7 +7445,7 @@
         </is>
       </c>
       <c r="B13" s="48" t="n">
-        <v>0.0457</v>
+        <v>0.043</v>
       </c>
       <c r="C13" s="49" t="inlineStr">
         <is>
@@ -7671,15 +7671,13 @@
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>FRED matched yield  (rating-tier index)</t>
-        </is>
-      </c>
-      <c r="B33" s="46" t="n">
-        <v>0.04969999999999999</v>
-      </c>
+          <t>FRED matched yield</t>
+        </is>
+      </c>
+      <c r="B33" s="53" t="n"/>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>FRED BAMLC0A2CAAEY — AA</t>
+          <t>No rating returned — FRED method not applicable</t>
         </is>
       </c>
     </row>
@@ -7720,11 +7718,11 @@
         </is>
       </c>
       <c r="B36" s="46" t="n">
-        <v>0.05110000000000001</v>
+        <v>0.0484</v>
       </c>
       <c r="C36" s="44" t="inlineStr">
         <is>
-          <t>Rf 4.57% + spread 0.54%</t>
+          <t>Rf 4.30% + spread 0.54%</t>
         </is>
       </c>
     </row>
@@ -7750,11 +7748,11 @@
         </is>
       </c>
       <c r="B38" s="48" t="n">
-        <v>0.0336</v>
+        <v>0.0242</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
-          <t>Default = average of 3 source(s) above — override freely</t>
+          <t>Default = average of 2 source(s) above — override freely</t>
         </is>
       </c>
     </row>
@@ -8190,10 +8188,10 @@
         <v>0.1466</v>
       </c>
       <c r="H7" s="71" t="n">
-        <v>0.0853</v>
+        <v>0.0834</v>
       </c>
       <c r="I7" s="71" t="n">
-        <v>0.067</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="J7" s="72">
         <f>I7</f>
@@ -8540,10 +8538,10 @@
         <v>477166.5</v>
       </c>
       <c r="H15" s="77" t="n">
-        <v>517850.9</v>
+        <v>516944.6</v>
       </c>
       <c r="I15" s="77" t="n">
-        <v>552549.1</v>
+        <v>553865.5</v>
       </c>
       <c r="J15" s="78">
         <f>I15*(1+J7)</f>
@@ -8576,22 +8574,22 @@
       </c>
       <c r="H16" s="82" t="inlineStr">
         <is>
-          <t>498,080 — 557,121</t>
+          <t>497,208 — 556,146</t>
         </is>
       </c>
       <c r="I16" s="82" t="inlineStr">
         <is>
-          <t>550,699 — 554,399</t>
+          <t>551,890 — 555,841</t>
         </is>
       </c>
       <c r="J16" s="82" t="inlineStr">
         <is>
-          <t>466,391 — 514,842</t>
+          <t>574,242 — 633,897</t>
         </is>
       </c>
       <c r="K16" s="82" t="inlineStr">
         <is>
-          <t>605,970 — 668,920</t>
+          <t>605,902 — 668,845</t>
         </is>
       </c>
       <c r="L16" s="83" t="inlineStr">
@@ -8738,10 +8736,10 @@
         <v>172226.1</v>
       </c>
       <c r="H20" s="77" t="n">
-        <v>186910.5</v>
+        <v>186583.4</v>
       </c>
       <c r="I20" s="77" t="n">
-        <v>199434.3</v>
+        <v>199909.4</v>
       </c>
       <c r="J20" s="78">
         <f>J15*J8</f>
@@ -8774,22 +8772,22 @@
       </c>
       <c r="H21" s="82" t="inlineStr">
         <is>
-          <t>179,774 — 201,085</t>
+          <t>179,460 — 200,733</t>
         </is>
       </c>
       <c r="I21" s="82" t="inlineStr">
         <is>
-          <t>198,766 — 200,102</t>
+          <t>199,196 — 200,623</t>
         </is>
       </c>
       <c r="J21" s="82" t="inlineStr">
         <is>
-          <t>168,337 — 185,824</t>
+          <t>207,264 — 228,795</t>
         </is>
       </c>
       <c r="K21" s="82" t="inlineStr">
         <is>
-          <t>218,716 — 241,437</t>
+          <t>218,691 — 241,409</t>
         </is>
       </c>
       <c r="L21" s="83" t="inlineStr">
@@ -9969,7 +9967,7 @@
         </is>
       </c>
       <c r="B61" s="111" t="n">
-        <v>310.3</v>
+        <v>312.51</v>
       </c>
       <c r="C61" s="103" t="n"/>
       <c r="D61" s="103" t="n"/>
@@ -10069,7 +10067,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="113" t="inlineStr">
         <is>
-          <t>JS SCORECARD — AAPL  |  Master Prompt v2  |  26 May 2026  |  Sector bucket: Tech Growth</t>
+          <t>JS SCORECARD — AAPL  |  Master Prompt v2  |  29 May 2026  |  Sector bucket: Tech Growth</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10584,7 @@
       </c>
       <c r="D22" s="129" t="inlineStr">
         <is>
-          <t>Fwd P/E 35.5x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.0x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=4.00 | fwd_pe=35.5x→4.00 | abs=1.5 → blended 40/40/20=3.50]  PEG=212.09 (fwd_pe=35.5x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
+          <t>Fwd P/E 35.7x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 21.1x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=3.90 | fwd_pe=35.7x→3.90 | abs=1.5 → blended 40/40/20=3.42]  PEG=213.29 (fwd_pe=35.7x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
         </is>
       </c>
       <c r="E22" s="136" t="inlineStr">
@@ -10595,7 +10593,7 @@
         </is>
       </c>
       <c r="F22" s="131" t="n">
-        <v>3.75</v>
+        <v>3.67</v>
       </c>
       <c r="G22" s="132">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10603,7 +10601,7 @@
       </c>
       <c r="H22" s="133" t="inlineStr">
         <is>
-          <t>Fwd P/E 35.5x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 20.0x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=4.00 | fwd_pe=35.5x→4.00 | abs=1.5 → blended 40/40/20=3.50]  PEG=212.09 (fwd_pe=35.5x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
+          <t>Fwd P/E 35.7x (scoring basis)  |  5yr avg 29.9x  |  Sector median 31.7x  |  DCF-implied 21.1x [ref only — not used as benchmark]  [+19% vs benchmark]  [trail=3.90 | fwd_pe=35.7x→3.90 | abs=1.5 → blended 40/40/20=3.42]  PEG=213.29 (fwd_pe=35.7x / eps_growth=17%)  [revision:Modest upgrade expected→+0.25]</t>
         </is>
       </c>
     </row>
@@ -10623,7 +10621,7 @@
       </c>
       <c r="D23" s="129" t="inlineStr">
         <is>
-          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.7x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=41.0x→0.11 | abs=4.0 → blended 40/40/20=1.29]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
+          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 24.0x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.10 | fwd_pfcf=41.3x→1.03 | abs=4.0 → blended 40/40/20=2.05]  [fcf_yield=2.6% vs rf=4.3%  spread=-1.7%→modifier=-0.25]</t>
         </is>
       </c>
       <c r="E23" s="134" t="inlineStr">
@@ -10632,7 +10630,7 @@
         </is>
       </c>
       <c r="F23" s="131" t="n">
-        <v>1.04</v>
+        <v>1.8</v>
       </c>
       <c r="G23" s="132">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10640,7 +10638,7 @@
       </c>
       <c r="H23" s="133" t="inlineStr">
         <is>
-          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 22.7x [ref only — not used as benchmark]  [+41% vs benchmark]  [trail=1.11 | fwd_pfcf=41.0x→0.11 | abs=4.0 → blended 40/40/20=1.29]  [fcf_yield=2.6% vs rf=4.6%  spread=-2.0%→modifier=-0.25]</t>
+          <t>Current 38.7x  |  5yr avg 29.2x  |  Sector median 27.5x  |  DCF-implied 24.0x [ref only — not used as benchmark]  [+33% vs benchmark]  [trail=2.10 | fwd_pfcf=41.3x→1.03 | abs=4.0 → blended 40/40/20=2.05]  [fcf_yield=2.6% vs rf=4.3%  spread=-1.7%→modifier=-0.25]</t>
         </is>
       </c>
     </row>

</xml_diff>